<commit_message>
Estandarizacion del generico 2, 21/05/2024
</commit_message>
<xml_diff>
--- a/Archivos/CONFIGURACION/Config.xlsx
+++ b/Archivos/CONFIGURACION/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Procesos_UiPath\00_GENERICOWindowsProcess_XX_XX_XX\Archivos\CONFIGURACION\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Procesos_UiPath\00_GENERICO_WINDOWS_NEGOCIOS_FINANCIEROS_XX_XX_XX\Archivos\CONFIGURACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11688C8E-F18B-4E72-BFE9-BE6ADD8E953C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40DE73E-8645-43D2-81CB-CC60AF1EFE74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="228">
   <si>
     <t>Name</t>
   </si>
@@ -817,6 +817,12 @@
   </si>
   <si>
     <t>00_GENERICO_WINDOWS_NEGOCIOS_FINANCIEROS_XX_XX_XX</t>
+  </si>
+  <si>
+    <t>C:\Users\USR\AppData\Local\Programs\Python\Python38\</t>
+  </si>
+  <si>
+    <t>C:\Program Files\Python38\</t>
   </si>
 </sst>
 </file>
@@ -1640,10 +1646,16 @@
       <c r="A12" s="2" t="s">
         <v>142</v>
       </c>
+      <c r="B12" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="13" spans="1:26" ht="14" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>143</v>
+      </c>
+      <c r="B13" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">

</xml_diff>